<commit_message>
Ember pull: drop Bangladesh, Sri Lanka, Thailand (monthly) and Bhutan (yearly) - all on raw feeds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BjcnPNGA6ZkWeQkXXc23hq
</commit_message>
<xml_diff>
--- a/output/Data and Chart Outputs/south_southeast_asia_power_by_type_annual.xlsx
+++ b/output/Data and Chart Outputs/south_southeast_asia_power_by_type_annual.xlsx
@@ -1,29 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Units" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Chart" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Chart - Myanmar" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Chart - Cambodia" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Chart - Laos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Chart - Brunei" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Chart - Nepal" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Chart - Bhutan" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Chart - Timor-Leste" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Indonesia" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Myanmar" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Cambodia" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Laos" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Brunei" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Nepal" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Bhutan" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Timor-Leste" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Units" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart - Myanmar" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart - Cambodia" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart - Laos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart - Brunei" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart - Nepal" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart - Timor-Leste" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indonesia" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Myanmar" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cambodia" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Laos" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brunei" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nepal" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timor-Leste" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,8 +31,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy"/>
+    <numFmt numFmtId="164" formatCode="yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -74,10 +72,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -155,13 +154,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -186,10 +185,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -214,10 +213,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -242,10 +241,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -270,10 +269,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EDA100"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -298,10 +297,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="E87BA4"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -326,10 +325,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="008300"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -354,10 +353,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="9A9A9A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -390,8 +389,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr rot="-2700000" vert="horz"/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -417,8 +416,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -435,7 +434,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -449,7 +448,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -458,13 +457,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -489,10 +488,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -517,10 +516,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -545,10 +544,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -573,10 +572,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EDA100"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -601,10 +600,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="E87BA4"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -629,10 +628,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="008300"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -657,10 +656,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="9A9A9A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -693,8 +692,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr rot="-2700000" vert="horz"/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -720,8 +719,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -738,7 +737,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -752,7 +751,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -761,13 +760,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -792,10 +791,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -820,10 +819,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -848,10 +847,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -876,10 +875,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EDA100"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -904,10 +903,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="E87BA4"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -932,10 +931,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="008300"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -960,10 +959,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="9A9A9A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -996,8 +995,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr rot="-2700000" vert="horz"/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1023,8 +1022,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1041,7 +1040,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1055,7 +1054,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -1064,13 +1063,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1095,10 +1094,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1123,10 +1122,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1151,10 +1150,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1179,10 +1178,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EDA100"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1207,10 +1206,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="E87BA4"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1235,10 +1234,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="008300"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1263,10 +1262,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="9A9A9A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1299,8 +1298,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr rot="-2700000" vert="horz"/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1326,8 +1325,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1344,7 +1343,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1358,7 +1357,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -1367,13 +1366,13 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1398,10 +1397,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1426,10 +1425,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1454,10 +1453,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1482,10 +1481,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EDA100"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1510,10 +1509,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="E87BA4"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1538,10 +1537,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="008300"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1566,10 +1565,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="9A9A9A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1602,8 +1601,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr rot="-2700000" vert="horz"/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1629,8 +1628,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1647,7 +1646,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1661,7 +1660,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -1670,13 +1669,13 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1701,10 +1700,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1729,10 +1728,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1757,10 +1756,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1785,10 +1784,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EDA100"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1813,10 +1812,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="E87BA4"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1841,10 +1840,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="008300"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1869,10 +1868,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="9A9A9A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1905,8 +1904,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr rot="-2700000" vert="horz"/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1932,8 +1931,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1950,7 +1949,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1964,7 +1963,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -1973,18 +1972,18 @@
 </file>
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Bhutan power generation by type (annual) (to 2024)</a:t>
+              <a:t>Timor-Leste power generation by type (annual) (to 2024)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -2000,26 +1999,26 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Chart - Bhutan'!B1</f>
+              <f>'Chart - Timor-Leste'!B1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Chart - Bhutan'!$A$2:$A$5</f>
+              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart - Bhutan'!$B$2:$B$5</f>
+              <f>'Chart - Timor-Leste'!$B$2:$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -2028,26 +2027,26 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Chart - Bhutan'!C1</f>
+              <f>'Chart - Timor-Leste'!C1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Chart - Bhutan'!$A$2:$A$5</f>
+              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart - Bhutan'!$C$2:$C$5</f>
+              <f>'Chart - Timor-Leste'!$C$2:$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -2056,26 +2055,26 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Chart - Bhutan'!D1</f>
+              <f>'Chart - Timor-Leste'!D1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Chart - Bhutan'!$A$2:$A$5</f>
+              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart - Bhutan'!$D$2:$D$5</f>
+              <f>'Chart - Timor-Leste'!$D$2:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -2084,26 +2083,26 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Chart - Bhutan'!E1</f>
+              <f>'Chart - Timor-Leste'!E1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="EDA100"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Chart - Bhutan'!$A$2:$A$5</f>
+              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart - Bhutan'!$E$2:$E$5</f>
+              <f>'Chart - Timor-Leste'!$E$2:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -2112,26 +2111,26 @@
           <order val="4"/>
           <tx>
             <strRef>
-              <f>'Chart - Bhutan'!F1</f>
+              <f>'Chart - Timor-Leste'!F1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="E87BA4"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Chart - Bhutan'!$A$2:$A$5</f>
+              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart - Bhutan'!$F$2:$F$5</f>
+              <f>'Chart - Timor-Leste'!$F$2:$F$5</f>
             </numRef>
           </val>
         </ser>
@@ -2140,26 +2139,26 @@
           <order val="5"/>
           <tx>
             <strRef>
-              <f>'Chart - Bhutan'!G1</f>
+              <f>'Chart - Timor-Leste'!G1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="008300"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Chart - Bhutan'!$A$2:$A$5</f>
+              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart - Bhutan'!$G$2:$G$5</f>
+              <f>'Chart - Timor-Leste'!$G$2:$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -2168,26 +2167,26 @@
           <order val="6"/>
           <tx>
             <strRef>
-              <f>'Chart - Bhutan'!H1</f>
+              <f>'Chart - Timor-Leste'!H1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="9A9A9A"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Chart - Bhutan'!$A$2:$A$5</f>
+              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart - Bhutan'!$H$2:$H$5</f>
+              <f>'Chart - Timor-Leste'!$H$2:$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -2208,8 +2207,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr rot="-2700000" vert="horz"/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -2235,8 +2234,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -2253,7 +2252,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2267,310 +2266,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln>
-      <a:noFill/>
-      <a:prstDash val="solid"/>
-    </a:ln>
-  </spPr>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Timor-Leste power generation by type (annual) (to 2024)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="0"/>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="stacked"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Chart - Timor-Leste'!B1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="2A78D6"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$B$2:$B$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Chart - Timor-Leste'!C1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="EB6834"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$C$2:$C$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'Chart - Timor-Leste'!D1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="1BAF7A"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$D$2:$D$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <strRef>
-              <f>'Chart - Timor-Leste'!E1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="EDA100"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$E$2:$E$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <tx>
-            <strRef>
-              <f>'Chart - Timor-Leste'!F1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="E87BA4"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$F$2:$F$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="5"/>
-          <order val="5"/>
-          <tx>
-            <strRef>
-              <f>'Chart - Timor-Leste'!G1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="008300"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$G$2:$G$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="6"/>
-          <order val="6"/>
-          <tx>
-            <strRef>
-              <f>'Chart - Timor-Leste'!H1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="9A9A9A"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$A$2:$A$5</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Chart - Timor-Leste'!$H$2:$H$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="30"/>
-        <overlap val="100"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="b"/>
-        <numFmt formatCode="yyyy" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="low"/>
-        <txPr>
-          <a:bodyPr rot="-2700000" vert="horz"/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </txPr>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-        <tickLblSkip val="1"/>
-        <tickMarkSkip val="1"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>GWh per year</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-          <overlay val="0"/>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-      <spPr>
-        <a:ln>
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </plotArea>
-    <legend>
-      <legendPos val="b"/>
-      <overlay val="0"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-  <spPr>
-    <a:ln>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -2579,7 +2275,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -2594,9 +2290,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2606,7 +2302,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -2621,9 +2317,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2633,7 +2329,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -2648,9 +2344,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2660,7 +2356,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -2675,9 +2371,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2687,7 +2383,7 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -2702,9 +2398,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2714,7 +2410,7 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -2729,9 +2425,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2741,7 +2437,7 @@
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -2756,36 +2452,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>9</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="10080000" cy="4680000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -3117,7 +2786,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
@@ -3128,11 +2796,10 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Yearly. Indonesia: 2021 to 2024; Myanmar: 2021 to 2024; Cambodia: 2021 to 2025; Laos: 2021 to 2024; Brunei: 2021 to 2024; Nepal: 2021 to 2024; Bhutan: 2021 to 2024; Timor-Leste: 2021 to 2024. Ember lags real time by one to several months (it varies by country); the weekly run picks up new months as they're released.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
+          <t>Yearly. Indonesia: 2021 to 2024; Myanmar: 2021 to 2024; Cambodia: 2021 to 2025; Laos: 2021 to 2024; Brunei: 2021 to 2024; Nepal: 2021 to 2024; Timor-Leste: 2021 to 2024. Ember lags real time by one to several months (it varies by country); the weekly run picks up new months as they're released.</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -3158,7 +2825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3189,30 +2856,35 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Nuclear_GWh</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Other Fossil_GWh</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Other Renewables_GWh</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Solar_GWh</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Wind_GWh</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Total_GWh</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Gas_for_power_est_mcm_per_day</t>
         </is>
@@ -3226,34 +2898,37 @@
         <v>2021</v>
       </c>
       <c r="C2" t="n">
-        <v>14960</v>
+        <v>260</v>
       </c>
       <c r="D2" t="n">
-        <v>189960</v>
+        <v>2120</v>
       </c>
       <c r="E2" t="n">
-        <v>56530</v>
+        <v>7880</v>
       </c>
       <c r="F2" t="n">
-        <v>24700</v>
+        <v>9510</v>
       </c>
       <c r="G2" t="n">
-        <v>6670</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>15910</v>
+        <v>120</v>
       </c>
       <c r="I2" t="n">
-        <v>190</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>440</v>
+        <v>90</v>
       </c>
       <c r="K2" t="n">
-        <v>309360</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>29.35</v>
+        <v>19980</v>
+      </c>
+      <c r="M2" t="n">
+        <v>4.09</v>
       </c>
     </row>
     <row r="3">
@@ -3264,34 +2939,37 @@
         <v>2022</v>
       </c>
       <c r="C3" t="n">
-        <v>20620</v>
+        <v>270</v>
       </c>
       <c r="D3" t="n">
-        <v>205310</v>
+        <v>2170</v>
       </c>
       <c r="E3" t="n">
-        <v>56710</v>
+        <v>11470</v>
       </c>
       <c r="F3" t="n">
-        <v>27300</v>
+        <v>9070</v>
       </c>
       <c r="G3" t="n">
-        <v>6110</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>16690</v>
+        <v>110</v>
       </c>
       <c r="I3" t="n">
-        <v>440</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>360</v>
+        <v>160</v>
       </c>
       <c r="K3" t="n">
-        <v>333540</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>29.44</v>
+        <v>23250</v>
+      </c>
+      <c r="M3" t="n">
+        <v>5.95</v>
       </c>
     </row>
     <row r="4">
@@ -3302,34 +2980,37 @@
         <v>2023</v>
       </c>
       <c r="C4" t="n">
-        <v>22480</v>
+        <v>270</v>
       </c>
       <c r="D4" t="n">
-        <v>216780</v>
+        <v>1120</v>
       </c>
       <c r="E4" t="n">
-        <v>62040</v>
+        <v>10040</v>
       </c>
       <c r="F4" t="n">
-        <v>24590</v>
+        <v>9430</v>
       </c>
       <c r="G4" t="n">
-        <v>6580</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>16940</v>
+        <v>130</v>
       </c>
       <c r="I4" t="n">
-        <v>710</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>480</v>
+        <v>110</v>
       </c>
       <c r="K4" t="n">
-        <v>350600</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>32.21</v>
+        <v>21100</v>
+      </c>
+      <c r="M4" t="n">
+        <v>5.21</v>
       </c>
     </row>
     <row r="5">
@@ -3340,34 +3021,37 @@
         <v>2024</v>
       </c>
       <c r="C5" t="n">
-        <v>21330</v>
+        <v>270</v>
       </c>
       <c r="D5" t="n">
-        <v>228430</v>
+        <v>1200</v>
       </c>
       <c r="E5" t="n">
-        <v>68780</v>
+        <v>10000</v>
       </c>
       <c r="F5" t="n">
-        <v>27290</v>
+        <v>10000</v>
       </c>
       <c r="G5" t="n">
-        <v>7120</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>16770</v>
+        <v>120</v>
       </c>
       <c r="I5" t="n">
-        <v>1350</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>470</v>
+        <v>120</v>
       </c>
       <c r="K5" t="n">
-        <v>371540</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>35.61</v>
+        <v>21710</v>
+      </c>
+      <c r="M5" t="n">
+        <v>5.18</v>
       </c>
     </row>
   </sheetData>
@@ -3381,7 +3065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3402,47 +3086,22 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Gas_GWh</t>
+          <t>Hydro_GWh</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Hydro_GWh</t>
+          <t>Other Fossil_GWh</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Nuclear_GWh</t>
+          <t>Solar_GWh</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Other Fossil_GWh</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Other Renewables_GWh</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Solar_GWh</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Wind_GWh</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
           <t>Total_GWh</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Gas_for_power_est_mcm_per_day</t>
         </is>
       </c>
     </row>
@@ -3454,37 +3113,22 @@
         <v>2021</v>
       </c>
       <c r="C2" t="n">
-        <v>260</v>
+        <v>50</v>
       </c>
       <c r="D2" t="n">
-        <v>2120</v>
+        <v>3460</v>
       </c>
       <c r="E2" t="n">
-        <v>7880</v>
+        <v>5040</v>
       </c>
       <c r="F2" t="n">
-        <v>9510</v>
+        <v>550</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>610</v>
       </c>
       <c r="H2" t="n">
-        <v>120</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>90</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>19980</v>
-      </c>
-      <c r="M2" t="n">
-        <v>4.09</v>
+        <v>9710</v>
       </c>
     </row>
     <row r="3">
@@ -3495,37 +3139,22 @@
         <v>2022</v>
       </c>
       <c r="C3" t="n">
-        <v>270</v>
+        <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>2170</v>
+        <v>3140</v>
       </c>
       <c r="E3" t="n">
-        <v>11470</v>
+        <v>5900</v>
       </c>
       <c r="F3" t="n">
-        <v>9070</v>
+        <v>350</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="H3" t="n">
-        <v>110</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>160</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>23250</v>
-      </c>
-      <c r="M3" t="n">
-        <v>5.95</v>
+        <v>10100</v>
       </c>
     </row>
     <row r="4">
@@ -3536,37 +3165,22 @@
         <v>2023</v>
       </c>
       <c r="C4" t="n">
-        <v>270</v>
+        <v>70</v>
       </c>
       <c r="D4" t="n">
-        <v>1120</v>
+        <v>7820</v>
       </c>
       <c r="E4" t="n">
-        <v>10040</v>
+        <v>4840</v>
       </c>
       <c r="F4" t="n">
-        <v>9430</v>
+        <v>50</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>820</v>
       </c>
       <c r="H4" t="n">
-        <v>130</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>110</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>21100</v>
-      </c>
-      <c r="M4" t="n">
-        <v>5.21</v>
+        <v>13600</v>
       </c>
     </row>
     <row r="5">
@@ -3577,37 +3191,48 @@
         <v>2024</v>
       </c>
       <c r="C5" t="n">
-        <v>270</v>
+        <v>80</v>
       </c>
       <c r="D5" t="n">
-        <v>1200</v>
+        <v>9430</v>
       </c>
       <c r="E5" t="n">
-        <v>10000</v>
+        <v>4370</v>
       </c>
       <c r="F5" t="n">
-        <v>10000</v>
+        <v>530</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1070</v>
       </c>
       <c r="H5" t="n">
-        <v>120</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>120</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>21710</v>
-      </c>
-      <c r="M5" t="n">
-        <v>5.18</v>
+        <v>15480</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C6" t="n">
+        <v>60</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10050</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5310</v>
+      </c>
+      <c r="F6" t="n">
+        <v>450</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1890</v>
+      </c>
+      <c r="H6" t="n">
+        <v>17760</v>
       </c>
     </row>
   </sheetData>
@@ -3621,7 +3246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3642,22 +3267,47 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Gas_GWh</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Hydro_GWh</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Nuclear_GWh</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>Other Fossil_GWh</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Other Renewables_GWh</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>Solar_GWh</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Wind_GWh</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>Total_GWh</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Gas_for_power_est_mcm_per_day</t>
         </is>
       </c>
     </row>
@@ -3672,19 +3322,34 @@
         <v>50</v>
       </c>
       <c r="D2" t="n">
-        <v>3460</v>
+        <v>11880</v>
       </c>
       <c r="E2" t="n">
-        <v>5040</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>550</v>
+        <v>32900</v>
       </c>
       <c r="G2" t="n">
-        <v>610</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>9710</v>
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>70</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>44900</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -3695,22 +3360,37 @@
         <v>2022</v>
       </c>
       <c r="C3" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D3" t="n">
-        <v>3140</v>
+        <v>12180</v>
       </c>
       <c r="E3" t="n">
-        <v>5900</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>350</v>
+        <v>38740</v>
       </c>
       <c r="G3" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>10100</v>
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>80</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>51040</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -3721,22 +3401,37 @@
         <v>2023</v>
       </c>
       <c r="C4" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="D4" t="n">
-        <v>7820</v>
+        <v>12180</v>
       </c>
       <c r="E4" t="n">
-        <v>4840</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>50</v>
+        <v>40000</v>
       </c>
       <c r="G4" t="n">
-        <v>820</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>13600</v>
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>80</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>52300</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3747,48 +3442,37 @@
         <v>2024</v>
       </c>
       <c r="C5" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="D5" t="n">
-        <v>9430</v>
+        <v>12180</v>
       </c>
       <c r="E5" t="n">
-        <v>4370</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>530</v>
+        <v>40000</v>
       </c>
       <c r="G5" t="n">
-        <v>1070</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>15480</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C6" t="n">
-        <v>60</v>
-      </c>
-      <c r="D6" t="n">
-        <v>10050</v>
-      </c>
-      <c r="E6" t="n">
-        <v>5310</v>
-      </c>
-      <c r="F6" t="n">
-        <v>450</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1890</v>
-      </c>
-      <c r="H6" t="n">
-        <v>17760</v>
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>90</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>52310</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3875,37 +3559,37 @@
         <v>2021</v>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>11880</v>
+        <v>1240</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>4420</v>
       </c>
       <c r="F2" t="n">
-        <v>32900</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>44900</v>
+        <v>5700</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="3">
@@ -3916,37 +3600,37 @@
         <v>2022</v>
       </c>
       <c r="C3" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>12180</v>
+        <v>1210</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>4340</v>
       </c>
       <c r="F3" t="n">
-        <v>38740</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>51040</v>
+        <v>5600</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="4">
@@ -3957,37 +3641,37 @@
         <v>2023</v>
       </c>
       <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1140</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4420</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
         <v>40</v>
       </c>
-      <c r="D4" t="n">
-        <v>12180</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>40000</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>52300</v>
+        <v>5600</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="5">
@@ -3998,37 +3682,37 @@
         <v>2024</v>
       </c>
       <c r="C5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>12180</v>
+        <v>1100</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>4400</v>
       </c>
       <c r="F5" t="n">
-        <v>40000</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>52310</v>
+        <v>5560</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>2.28</v>
       </c>
     </row>
   </sheetData>
@@ -4118,34 +3802,34 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>1240</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>4420</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>9530</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L2" t="n">
-        <v>5700</v>
+        <v>9630</v>
       </c>
       <c r="M2" t="n">
-        <v>2.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -4159,34 +3843,34 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>1210</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>4340</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>10590</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L3" t="n">
-        <v>5600</v>
+        <v>10700</v>
       </c>
       <c r="M3" t="n">
-        <v>2.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -4200,34 +3884,34 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>1140</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>4420</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>10590</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L4" t="n">
-        <v>5600</v>
+        <v>10700</v>
       </c>
       <c r="M4" t="n">
-        <v>2.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -4241,34 +3925,34 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>4400</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>11000</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
+        <v>120</v>
+      </c>
+      <c r="K5" t="n">
         <v>10</v>
       </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
       <c r="L5" t="n">
-        <v>5560</v>
+        <v>11130</v>
       </c>
       <c r="M5" t="n">
-        <v>2.28</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4277,486 +3961,6 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Bioenergy_GWh</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Coal_GWh</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Gas_GWh</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Hydro_GWh</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Nuclear_GWh</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Other Fossil_GWh</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Other Renewables_GWh</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Solar_GWh</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Wind_GWh</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Total_GWh</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Gas_for_power_est_mcm_per_day</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>0</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>9530</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>90</v>
-      </c>
-      <c r="K2" t="n">
-        <v>10</v>
-      </c>
-      <c r="L2" t="n">
-        <v>9630</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>10590</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>100</v>
-      </c>
-      <c r="K3" t="n">
-        <v>10</v>
-      </c>
-      <c r="L3" t="n">
-        <v>10700</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>10590</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>100</v>
-      </c>
-      <c r="K4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L4" t="n">
-        <v>10700</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>11000</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>120</v>
-      </c>
-      <c r="K5" t="n">
-        <v>10</v>
-      </c>
-      <c r="L5" t="n">
-        <v>11130</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Bioenergy_GWh</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Coal_GWh</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Gas_GWh</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Hydro_GWh</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Nuclear_GWh</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Other Fossil_GWh</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Other Renewables_GWh</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Solar_GWh</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Wind_GWh</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Total_GWh</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Gas_for_power_est_mcm_per_day</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>0</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>10820</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>10820</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>10770</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>10770</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>11160</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>11160</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>11000</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>11000</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5051,7 +4255,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>44197</v>
       </c>
       <c r="B2" t="n">
@@ -5077,7 +4281,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>44562</v>
       </c>
       <c r="B3" t="n">
@@ -5103,7 +4307,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>44927</v>
       </c>
       <c r="B4" t="n">
@@ -5129,7 +4333,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>45292</v>
       </c>
       <c r="B5" t="n">
@@ -5215,7 +4419,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>44197</v>
       </c>
       <c r="B2" t="n">
@@ -5241,7 +4445,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>44562</v>
       </c>
       <c r="B3" t="n">
@@ -5267,7 +4471,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>44927</v>
       </c>
       <c r="B4" t="n">
@@ -5293,7 +4497,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>45292</v>
       </c>
       <c r="B5" t="n">
@@ -5379,7 +4583,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>44197</v>
       </c>
       <c r="B2" t="n">
@@ -5405,7 +4609,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>44562</v>
       </c>
       <c r="B3" t="n">
@@ -5431,7 +4635,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>44927</v>
       </c>
       <c r="B4" t="n">
@@ -5457,7 +4661,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>45292</v>
       </c>
       <c r="B5" t="n">
@@ -5483,7 +4687,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="3" t="n">
         <v>45658</v>
       </c>
       <c r="B6" t="n">
@@ -5569,7 +4773,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>44197</v>
       </c>
       <c r="B2" t="n">
@@ -5595,7 +4799,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>44562</v>
       </c>
       <c r="B3" t="n">
@@ -5621,7 +4825,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>44927</v>
       </c>
       <c r="B4" t="n">
@@ -5647,7 +4851,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>45292</v>
       </c>
       <c r="B5" t="n">
@@ -5733,7 +4937,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>44197</v>
       </c>
       <c r="B2" t="n">
@@ -5759,7 +4963,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>44562</v>
       </c>
       <c r="B3" t="n">
@@ -5785,7 +4989,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>44927</v>
       </c>
       <c r="B4" t="n">
@@ -5811,7 +5015,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>45292</v>
       </c>
       <c r="B5" t="n">
@@ -5897,7 +5101,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>44197</v>
       </c>
       <c r="B2" t="n">
@@ -5923,7 +5127,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>44562</v>
       </c>
       <c r="B3" t="n">
@@ -5949,7 +5153,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>44927</v>
       </c>
       <c r="B4" t="n">
@@ -5975,7 +5179,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>45292</v>
       </c>
       <c r="B5" t="n">
@@ -6061,11 +5265,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>44197</v>
       </c>
       <c r="B2" t="n">
-        <v>10820</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -6083,15 +5287,15 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>510</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>44562</v>
       </c>
       <c r="B3" t="n">
-        <v>10770</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -6109,15 +5313,15 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>510</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>44927</v>
       </c>
       <c r="B4" t="n">
-        <v>11160</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -6135,15 +5339,15 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>510</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>45292</v>
       </c>
       <c r="B5" t="n">
-        <v>11000</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -6161,7 +5365,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>510</v>
       </c>
     </row>
   </sheetData>
@@ -6176,160 +5380,219 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Hydro</t>
+          <t>Year</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Gas</t>
+          <t>Bioenergy_GWh</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Wind</t>
+          <t>Coal_GWh</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Gas_GWh</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Coal</t>
+          <t>Hydro_GWh</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Nuclear</t>
+          <t>Other Fossil_GWh</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Other Renewables_GWh</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Solar_GWh</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Wind_GWh</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Total_GWh</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Gas_for_power_est_mcm_per_day</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>44197</v>
+      <c r="A2" t="n">
+        <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>2021</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>14960</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>189960</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>56530</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>24700</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>6670</v>
       </c>
       <c r="H2" t="n">
-        <v>510</v>
+        <v>15910</v>
+      </c>
+      <c r="I2" t="n">
+        <v>190</v>
+      </c>
+      <c r="J2" t="n">
+        <v>440</v>
+      </c>
+      <c r="K2" t="n">
+        <v>309360</v>
+      </c>
+      <c r="L2" t="n">
+        <v>29.35</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>44562</v>
+      <c r="A3" t="n">
+        <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>2022</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>20620</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>205310</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>56710</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>27300</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>6110</v>
       </c>
       <c r="H3" t="n">
-        <v>510</v>
+        <v>16690</v>
+      </c>
+      <c r="I3" t="n">
+        <v>440</v>
+      </c>
+      <c r="J3" t="n">
+        <v>360</v>
+      </c>
+      <c r="K3" t="n">
+        <v>333540</v>
+      </c>
+      <c r="L3" t="n">
+        <v>29.44</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>44927</v>
+      <c r="A4" t="n">
+        <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>2023</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>22480</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>216780</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>62040</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>24590</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>6580</v>
       </c>
       <c r="H4" t="n">
-        <v>510</v>
+        <v>16940</v>
+      </c>
+      <c r="I4" t="n">
+        <v>710</v>
+      </c>
+      <c r="J4" t="n">
+        <v>480</v>
+      </c>
+      <c r="K4" t="n">
+        <v>350600</v>
+      </c>
+      <c r="L4" t="n">
+        <v>32.21</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>45292</v>
+      <c r="A5" t="n">
+        <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>2024</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>21330</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>228430</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>68780</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>27290</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>7120</v>
       </c>
       <c r="H5" t="n">
-        <v>510</v>
+        <v>16770</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1350</v>
+      </c>
+      <c r="J5" t="n">
+        <v>470</v>
+      </c>
+      <c r="K5" t="n">
+        <v>371540</v>
+      </c>
+      <c r="L5" t="n">
+        <v>35.61</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>